<commit_message>
refactoring dell'architettura da MVC a MVP
</commit_message>
<xml_diff>
--- a/bandi_estratti_totale.xlsx
+++ b/bandi_estratti_totale.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,17 +466,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://fornitori.cellnextelecom.it/albo/login</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>failed_error</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CELLNEXTELECOM</t>
+          <t>AUTOSTRADE</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -513,17 +513,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://fastweb.risk.coupahost.com/Account/Login</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>failed_creds</t>
+          <t>failed_error</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FASTWEB</t>
+          <t>AUTOSTRADE</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -560,7 +560,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://fastweb.risk.coupahost.com/Account/Login</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>FASTWEB</t>
+          <t>AUTOSTRADE</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -607,17 +607,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://fastweb.risk.coupahost.com/Account/Login</t>
+          <t>https://eprocurement.raiway.it/PortaleAppalti/it/homepage.wp</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>failed_creds</t>
+          <t>failed_error</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>FASTWEB</t>
+          <t>RAIWAY</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -654,7 +654,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://supplier.coupahost.com/sessions/new</t>
+          <t>https://www.edison.it/it/diventa-fornitore</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -664,7 +664,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SUPPLIER</t>
+          <t>EDISON</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -701,17 +701,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://fastweb.coupahost.com/sessions/supplier_login</t>
+          <t>https://www.anticorruzione.it/per-le-imprese</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>failed_error</t>
+          <t>success</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>FASTWEB</t>
+          <t>ANTICORRUZIONE</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -748,7 +748,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://fastweb.coupahost.com/sessions/supplier_login</t>
+          <t>https://atlantefotg.my.site.com/vendorportal/s/</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>FASTWEB</t>
+          <t>ATLANTEFOTG</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -795,7 +795,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://fastweb.coupahost.com/sessions/supplier_login</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>FASTWEB</t>
+          <t>AUTOSTRADE</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -842,27 +842,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://fastweb.coupahost.com/sessions/supplier_login</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>failed_error</t>
+          <t>success</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>FASTWEB</t>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Nessun bando estratto o login fallito</t>
+          <t>Gara europea a procedura aperta per il Servizio di raccolta, trasporto, consegna alle sale conta e contazione dei valori depositati presso le stazioni autostradali o altri siti ubicati nel territorio di competenza di ogni Direzione di Tronco di Autostrade</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 12:00</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Servizi</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -882,34 +882,34 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://fastweb.coupahost.com/sessions/supplier_login</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>failed_error</t>
+          <t>success</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>FASTWEB</t>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Nessun bando estratto o login fallito</t>
+          <t>COE_Fornitura di Cloruro di Calcio per le Direzioni di Tronco di ASPI</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10/06/2026 12:00</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -919,7 +919,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Forniture</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -929,14 +929,14 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://deiplus.build.it/index.php</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -946,17 +946,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>DEIPLUS</t>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Nessun bando estratto o login fallito</t>
+          <t>RDA 458591 - CTA RIQUALIFICA BS T1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>15/06/2026 23:59</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Servizi</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -976,34 +976,34 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://myaccount.ericsson.net/xpra/#/home</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>failed_captcha</t>
+          <t>success</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MYACCOUNT</t>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Nessun bando estratto o login fallito</t>
+          <t>Servizio di prove di laboratorio e indagini in sito, indagini geognostiche e rilievi topografici</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>17/06/2026 12:00</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Servizi</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
     </row>
@@ -1035,22 +1035,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>failed_error</t>
+          <t>success</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AUTOSTRADE</t>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Nessun bando estratto o login fallito</t>
+          <t>GARA EUROPEA A PROCEDURA APERTA PER IL SERVIZIO MANUTENTIVO DEGLI IMPIANTI DI ESAZIONE DI PEDAGGIO, DI VIABILITA', DI INFRASTRUTTURE ED ELETTRICI, COMPRENSIVO DI FORNITURA ACCESSORIA DI PARTI DI RICAMBIO.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>17/06/2026 18:00</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Servizi</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
     </row>
@@ -1082,22 +1082,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>failed_error</t>
+          <t>success</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AUTOSTRADE</t>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Nessun bando estratto o login fallito</t>
+          <t>APN_Servizio cablaggio impianti di esazione svincolo Maddaloni - A30</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>30/06/2026 12:00</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Servizi</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
     </row>
@@ -1129,22 +1129,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>failed_error</t>
+          <t>success</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AUTOSTRADE</t>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Nessun bando estratto o login fallito</t>
+          <t>903832_S.U. - Supporto idrodemolizioni nell'ambito degli interventi in somma urgenza del ponte di scolo Calcarata km. 23+991 nei tratti di competenza della Direzione 3^ Tronco Bologna</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>30/06/2026 23:00</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Servizi</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1164,34 +1164,34 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://a4mobility-appalti.maggiolicloud.it/PortaleAppalti/it/ppcommon_area_personale.wp?redirectflag=1</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>failed_manual</t>
+          <t>success</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>A4MOBILITY-APPALTI</t>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Nessun bando estratto o login fallito</t>
+          <t>S.U. - DT 5 - SERVIZI DI INGEGNERIA Direzione lavori e CSE per interventi su op. Idraul. N. 241</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>30/06/2026 23:59</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Servizi</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1211,34 +1211,34 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://www2.autostrade.it/</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>failed_manual</t>
+          <t>success</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>WWW2</t>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Nessun bando estratto o login fallito</t>
+          <t>Procedura aperta ex art. 71 D.Lgs. 36/2023_Acquisto licenze Microsoft MPSA 2026-29</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>01/07/2026 12:00</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Forniture</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1258,34 +1258,34 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://fastweb.risk.coupahost.com/Dashboard/Home</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>failed_creds</t>
+          <t>success</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>FASTWEB</t>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Nessun bando estratto o login fallito</t>
+          <t>PROCEDURA APERTA PER L’AFFIDAMENTO DELLA FORNITURA DI ROUTER CISCO DI BACKBONE PER I TRONCHI E DI ROUTER CISCO GEOGRAFICI PER LE STAZIONI, AREE DI SERVIZIO, SHELTER E GALLERIE SITUATI SULLE TRATTE AUTOSTRADALI DI COMPETENZA DI AUTOSTRADE PER L’ITALIA S.P.A</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>01/07/2026 12:00</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Forniture</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1305,14 +1305,14 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://imprese.istat.it/</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1322,17 +1322,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>IMPRESE</t>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Nessun bando estratto o login fallito</t>
+          <t>ESE_PROCEDURA APERTA PER L’APPALTO DEI SERVIZI MECCANIZZATI DI SGOMBERO NEVE E TRATTAMENTO ANTIGHIACCIO DA ESEGUIRSI LUNGO LE TRATTE AUTOSTRADALI DI COMPETENZA DELLA DIREZIONE 8° TRONCO DI BARI  (A16 - P.N. CANDELA, P.N. CERIGNOLA, P.N. CANOSA)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>01/07/2026 16:00</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Servizi</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1352,14 +1352,14 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://portaleacquisti.terna.it</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1369,17 +1369,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>PORTALETERNA</t>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Nessun bando estratto o login fallito</t>
+          <t>ESE_GARA EUROPEA A PROCEDURA APERTA PER L’AFFIDAMENTO DI MANUTENZIONEORDINARIA PROGRAMMATA ED INTERVENTI STRAORDINARI DI RIPRISTINO FUNZIONALITÀ DEGLI IMPIANTI DI STOCCAGGIO CLORURI PER DISGELO STRADALE</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>06/07/2026 16:00</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Servizi</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1399,30 +1399,34 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>www.anticorruzione.it</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>failed_error</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Nessun bando estratto o login fallito</t>
+          <t>TES_Servizio taratura e manutenzione delle apparecchiature PENETROMETRO e REOMETRO</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>08/07/2026 18:00</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1432,7 +1436,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Servizi</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1442,7 +1446,1942 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Negoziata ai sensi dell’art. 76 comma 4 lett. b del D.lgs. 36/2023
+TES_Fornitura SUMMS 5 e manutenzione triennale WDM</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>10/07/2026 00:00</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Forniture</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>TES_Fornitura n. 2 mezzi Ecodyn, misura della retroriflessione della segnaletica orizzontale e contratto di manutenzione</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>10/07/2026 14:00</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>L.i.Fe srl- aff. diretto- prove su mat. da costruzione - Galleria Monte Mario - A1-tratta Casalecchio di Reno – Sasso Marconi</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>30/09/2026 00:00</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Affidamento diretto Speri S.p.A - VAL4- tratte di competenza DT2, DT5 e DT7</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>31/10/2026 12:00</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>459056_ INCARICO DI SERVIZI DI INGEGNERIA PER INTERVENTO DI SOMMA URGENZA DI RIPRISTINO PONTE ADIGE KM 72+249 NEL TRATTO DI COMPETENZA DELLA DIREZIONE 3^ TRONCO DI BOLOGNA</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>31/10/2026 12:00</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>904083 - DT03/TEC
+904083 - DT3 - Somma Urgenza Alluvione 18 e 19 Settembre 2024 - Ripristino treansitabilità A14 tra le progressive 92+000 e 118+000  e D14 (Diramazione Ravenna) - Rimozione Fanghi.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>31/12/2026 14:00</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>451778 - DT03/TECNICA
+451778 - Intervento di Somma Urgenza per il ripristino dei gravi eventi alluvionali del 19 e 20 Ottobre 2024 - Pulizia Fabbricati. Ripristino delle funzionalità e della salubrità delle unità immobiliari di pertinenza DT3.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>31/12/2026 14:00</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>452833 - DT03/TEC
+452833 - Servizio di supporto al coordinatore per la sicurezza in fase di esecuzione per aspetti geotecnici e strutturali per l’intervento di somma urgenza di ripristino a seguito dei gravi eventi alluvionali del 18 e 19 settembre 2024.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>31/12/2026 14:00</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>904359 - DT03/Tecnica
+904359 - Somma Urgenza 18 e 19 Sett_2024 - A14 Intervento di ripristino Segnaletica Orizzontale.</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>31/12/2026 18:00</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Lavori</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>456913_S.U. INTERVENTO DI SOMMA URGENZA DI RIPRISTINO A SEGUITO DEI GRAVI EVENTI ALLUVIONALI DEL 18 E 19 SETTEMBRE 2024_ SPURGO OPERE IDRAULICHE</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>31/12/2026 20:00</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>GST S.N.C. - Assistenza topografica nell'ambito del progetto A1 MILANO - NAPOLI Tratto Modena – Brennero (A22)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>24/02/2027 23:59</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Ing. Gilbo - Servizio di collaudo statico - Tunnel subportuale Genova</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>01/05/2027 23:59</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>446747 - DT3/TEC
+446747 - Somma Urgenza per il ripristino del Ponte Scolo Calcarata km 23+991 - A13 Bologna - Padova - Prove di Laboratorio</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>31/12/2027 14:00</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Aff. diretto - Ing. Caputo - Viadotto Paolo e Omero - Collaudo Statico - RdA 455916</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>17/03/2028 12:00</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>904625 - DT3/TECNICA
+904625 - Intervento di somma urgenza a seguito dei gravi eventi alluvionali del 18 e 19 settembre 2024 - Ripristino smottamenti localizzati in A14. Fornitura e posa in opera palancole.</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>31/12/2028 12:00</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Lavori</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>ASA-DT3-TEC-462866 -SU RIPRISTINO GIUNTO LAMELLARE PONTE RENO - PE - DL - CSE</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>29/01/2029 15:00</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>ASA-DT3-TEC-904930 - DT3-TEC - A1 SOMMA URGENZA GIUNTO LAMELLARE PONTE RENO</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>29/01/2029 15:00</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Lavori</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>AERTECNO s.r.l. - Servizio di Servizio di assistenza topografica - Opere complementari di Pesaro - Altre bretelle</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>16/02/2030 23:29</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>DT3_somma urgenza per intervento di messa in sicurezza e ripristino delle condizioni di transitabilità dell’Autostrada A14 tra le progr. Km 92+000 e km 118+000 e la D14 a seguito degli eventi alluvionali del 18 e 19 settembre 2024</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>23/05/2030 00:00</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Lavori</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Avvisi di gara procedure non telematiche (2017-2021) vecchio portale NGA</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>01/06/2030 00:00</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Lavori</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>DT3 - COD. APP. 021/BO/2024 SOMMA URGENZA 19-20 OTTOBRE 2024 - LAVORI FORNITURA E POSA PALANCOLE</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>04/06/2030 12:00</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Lavori</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>S.U.- INTERVENTI DI RISPRISTINO A SEGUITO DI ALLUVIONE 19 E 20 OTTOBRE 2024 - DT3 - COLLAUDO STATICO</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>21/08/2030 12:00</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Avviso istituzione Albo Fornitori</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>01/09/2030 00:00</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Altro</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>451161 DT3-RIPRISTINO IMP. CLIMATIZZAZIONE-SU/EVENTI ALLUVIONALI 18/19 SET.2024</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>10/11/2030 00:00</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>452711 DT3-SUPPORTO DL-SU/EVENTI ALLUVIONALI 18/19 SET.2024</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>10/11/2030 12:00</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>SOMMA URGENZA DI RIPRISTINO PONTE ADIGE KM 72+249 - INSTALLAZIONE CANTIERIZZAZIONE, GUARDIANIA E SEGNALAMENTO ACCODAMENTI IN AMBITO AUTOSTRADALE - DT3</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>11/11/2030 09:00</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Avviso istituzione nuova sezione Albo Fornitori - Servizi di ingegneria</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>31/12/2030 00:00</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Altro</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ASA - DT3-TEC - 459054 - SU PONTE ADIGE KM 72+249 - FORNITURA MAT. SISTEMI PRECOMPRESSIONE</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>16/01/2031 14:00</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Forniture</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>904671 - SOMMA URGENZA PER RIPRISTINO SISTEMI DI PRECOMPRESSIONE PONTE ADIGE KM 72+249</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>26/01/2031 14:00</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Lavori</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>ASA - DT3-TEC - 456119 - SU OTT 2024  - Fornitura barriere New Jersey ET 100</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>30/01/2031 14:00</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Forniture</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>ASA-DT3-TEC 453151 - CST PER SU EVENTI ALLUVIONALI DEL 19 E 20 OTTOBRE 2024</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>06/02/2031 15:00</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>ASA - DT3-TEC - 459055 - SU PONTE ADIGE KM 72+249 - INDAGINI E PROVE DI LABORATORIO</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>16/02/2031 14:00</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>904754_Intervento in somma urgenza per la messa in sicurezza del fabbricato e pensiline della stazione di Roma Ovest a seguito di incendio di un veicolo presente in pista</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>31/03/2031 23:00</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Lavori</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>ARAN PROGETTI S.R.L. - Servizio di sorveglianza archeologica - Progetti speciali Liguria Lotto A e Lotto B</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>07/04/2031 23:59</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>ASA - DT3 - TEC - 905067 - A14 SU SETT. 2024_SEGNALETICA CANT. E NJ</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>14/04/2031 14:00</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Lavori</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>ASA - DT3 - TEC - 904994 - SU OTTORE 2024 - PALANCOLE</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>17/04/2031 14:00</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Lavori</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>443718 - DT03/TEC
+443718 - DT3 - Somma Urgenza Cavalcavia Occhiobello A13 - Installazione cantierizzazione, guardiania e regolazione dei flussi veicolari.</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>31/12/2031 14:00</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>455277_S.U._Incarico di progettazione e  Coordinamento della Sicurezza in fase di progettazione nell'ambito degli interventi sull'OP. 241 km.624.728  N.- DT5</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>31/12/2035 12:00</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Servizi</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Istruzioni Fatturazione Elettronica</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>21/12/2099 12:00</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Altro</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Avviso pubblico Nuovo Regolamento Albo Fornitori 2021</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>31/12/2099 00:00</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Altro</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>AUTOSTRADE PER L'ITALIA SPA</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Nuovo Albo Fornitori del Gruppo Autostrade</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>31/12/2999 12:00</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Altro</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>https://autostrade.bravosolution.com/web/login.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
versione CORE completa, vedere gli md limiti, documentazione e read me per maggiori informazioni
</commit_message>
<xml_diff>
--- a/bandi_estratti_totale.xlsx
+++ b/bandi_estratti_totale.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,27 +466,23 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.acquistionlinerfi.it/web/error.html?_ncp=1753696951455.127431-1</t>
+          <t>eprocurement.gruppofs.it</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>success</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>RETE FERROVIARIA ITALIANA</t>
-        </is>
-      </c>
+          <t>failed_error</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DAC.0186.2026_Fornitura di "PALI TE"</t>
+          <t>Nessun bando estratto o login fallito</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>15/06/2026</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -496,17 +492,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Fornitura</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Fornitura di "PALI TE"</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.acquistionlinerfi.it/web/error.html?_ncp=1753696951455.127431-1</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -523,17 +519,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>RETE FERROVIARIA ITALIANA</t>
+          <t>ACQUISTIONLINERFI</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>DAC.326.2026 - Servizio per interventi su chiamata e programmati per pulizia, rimozione detriti su pile dei ponti dei fiumi ricadenti nella giurisdizione della Direzione Operativa Infrastrutture Milano</t>
+          <t>DAC.0186.2026_Fornitura di "PALI TE"</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>17/06/2026</t>
+          <t>15/06/2026 12:00</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -543,17 +539,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Servizi</t>
+          <t>Fornitura</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Servizio per interventi su chiamata e programmati per pulizia, rimozione detriti su pile dei ponti dei fiumi ricadenti nella giurisdizione della Direzione Operativa Infrastrutture Milano</t>
+          <t>Rete Ferroviaria Italiana</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://www.acquistionlinerfi.it/web/error.html?_ncp=1753696951455.127431-1</t>
+          <t>https://www.acquistionlinerfi.it/esop/toolkit/opportunity/current/list.si?reset=true&amp;resetstored=true&amp;customLoginPage=%2Fweb%2Flogin.html&amp;_ncp=1781183967356.1684912-1#fh</t>
         </is>
       </c>
     </row>
@@ -570,17 +566,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>RETE FERROVIARIA ITALIANA</t>
+          <t>ACQUISTIONLINERFI</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>DAC.0317.2026_GPA_Servizio di manutenzione attrezzature e macchinari dell’Officina Nazionale Mezzi d’Opera</t>
+          <t>DAC.326.2026 - Servizio per interventi su chiamata e programmati per pulizia, rimozione detriti su pile dei ponti dei fiumi ricadenti nella giurisdizione della Direzione Operativa Infrastrutture Milano</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>17/06/2026 12:00</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -595,12 +591,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Servizio di manutenzione attrezzature e macchinari dell’Officina Nazionale Mezzi d’Opera</t>
+          <t>Rete Ferroviaria Italiana</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://www.acquistionlinerfi.it/web/error.html?_ncp=1753696951455.127431-1</t>
+          <t>https://www.acquistionlinerfi.it/esop/toolkit/opportunity/current/list.si?reset=true&amp;resetstored=true&amp;customLoginPage=%2Fweb%2Flogin.html&amp;_ncp=1781183967356.1684912-1#fh</t>
         </is>
       </c>
     </row>
@@ -617,17 +613,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>RETE FERROVIARIA ITALIANA</t>
+          <t>ACQUISTIONLINERFI</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>DAC.0211.2026 - Key Management System</t>
+          <t>DAC.0317.2026_GPA_Servizio di manutenzione attrezzature e macchinari dell’Officina Nazionale Mezzi d’Opera</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>19/06/2026</t>
+          <t>18/06/2026 12:00</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -642,12 +638,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Key Management System</t>
+          <t>Rete Ferroviaria Italiana</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://www.acquistionlinerfi.it/web/error.html?_ncp=1753696951455.127431-1</t>
+          <t>https://www.acquistionlinerfi.it/esop/toolkit/opportunity/current/list.si?reset=true&amp;resetstored=true&amp;customLoginPage=%2Fweb%2Flogin.html&amp;_ncp=1781183967356.1684912-1#fh</t>
         </is>
       </c>
     </row>
@@ -664,17 +660,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>RETE FERROVIARIA ITALIANA</t>
+          <t>ACQUISTIONLINERFI</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>DAC.0010.2026 - GPA Multilotto Fornitura, in regime di Full Maintenance Service, dei Caricatori Strada Rotaia pesanti</t>
+          <t>DAC.0211.2026 - Key Management System</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>22/06/2026</t>
+          <t>19/06/2026 12:00</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -684,17 +680,17 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Fornitura</t>
+          <t>Servizi</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Fornitura, in regime di Full Maintenance Service, dei Caricatori Strada Rotaia pesanti</t>
+          <t>Rete Ferroviaria Italiana</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://www.acquistionlinerfi.it/web/error.html?_ncp=1753696951455.127431-1</t>
+          <t>https://www.acquistionlinerfi.it/esop/toolkit/opportunity/current/list.si?reset=true&amp;resetstored=true&amp;customLoginPage=%2Fweb%2Flogin.html&amp;_ncp=1781183967356.1684912-1#fh</t>
         </is>
       </c>
     </row>
@@ -711,17 +707,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>RETE FERROVIARIA ITALIANA</t>
+          <t>ACQUISTIONLINERFI</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DAC.0193.2026_Fornitura di Attrezzaggio TE</t>
+          <t>DAC.0010.2026 - GPA Multilotto Fornitura, in regime di Full Maintenance Service, dei Caricatori Strada Rotaia pesanti</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>22/06/2026</t>
+          <t>22/06/2026 12:00</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -736,12 +732,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Fornitura di Attrezzaggio TE</t>
+          <t>Rete Ferroviaria Italiana</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://www.acquistionlinerfi.it/web/error.html?_ncp=1753696951455.127431-1</t>
+          <t>https://www.acquistionlinerfi.it/esop/toolkit/opportunity/current/list.si?reset=true&amp;resetstored=true&amp;customLoginPage=%2Fweb%2Flogin.html&amp;_ncp=1781183967356.1684912-1#fh</t>
         </is>
       </c>
     </row>
@@ -758,17 +754,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>RETE FERROVIARIA ITALIANA</t>
+          <t>ACQUISTIONLINERFI</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>DAC.0006.2026 - GPA Multilotto Fornitura, in regime di Full Maintenance Service, di Carri Tramoggia da 20 m3</t>
+          <t>DAC.0193.2026_Fornitura di Attrezzaggio TE</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>23/06/2026</t>
+          <t>22/06/2026 12:00</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -783,12 +779,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>GPA Multilotto Fornitura, in regime di Full Maintenance Service, di Carri Tramoggia da 20 m3</t>
+          <t>Rete Ferroviaria Italiana</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://www.acquistionlinerfi.it/web/error.html?_ncp=1753696951455.127431-1</t>
+          <t>https://www.acquistionlinerfi.it/esop/toolkit/opportunity/current/list.si?reset=true&amp;resetstored=true&amp;customLoginPage=%2Fweb%2Flogin.html&amp;_ncp=1781183967356.1684912-1#fh</t>
         </is>
       </c>
     </row>
@@ -805,17 +801,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>RETE FERROVIARIA ITALIANA</t>
+          <t>ACQUISTIONLINERFI</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>DAC.0008.2026 - Fornitura, in regime di Full Maintenance Service, di Stabilizzatrici da utilizzare per il mantenimento in efficienza dell’Infrastruttura Ferroviaria Nazionale</t>
+          <t>DAC.0006.2026 - GPA Multilotto Fornitura, in regime di Full Maintenance Service, di Carri Tramoggia da 20 m3</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>26/06/2026</t>
+          <t>23/06/2026 12:00</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -830,12 +826,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Fornitura, in regime di Full Maintenance Service, di Stabilizzatrici da utilizzare per il mantenimento in efficienza dell’Infrastruttura Ferroviaria Nazionale</t>
+          <t>Rete Ferroviaria Italiana</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://www.acquistionlinerfi.it/web/error.html?_ncp=1753696951455.127431-1</t>
+          <t>https://www.acquistionlinerfi.it/esop/toolkit/opportunity/current/list.si?reset=true&amp;resetstored=true&amp;customLoginPage=%2Fweb%2Flogin.html&amp;_ncp=1781183967356.1684912-1#fh</t>
         </is>
       </c>
     </row>
@@ -852,17 +848,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>RETE FERROVIARIA ITALIANA</t>
+          <t>ACQUISTIONLINERFI</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>DAC.0111.2026_Fornitura di SALDATURE ALLUMINOTERMICHE</t>
+          <t>DAC.0008.2026 - Fornitura, in regime di Full Maintenance Service, di Stabilizzatrici da utilizzare per il mantenimento in efficienza dell’Infrastruttura Ferroviaria Nazionale</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>29/06/2026</t>
+          <t>26/06/2026 12:00</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -877,12 +873,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Fornitura di SALDATURE ALLUMINOTERMICHE</t>
+          <t>Rete Ferroviaria Italiana</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://www.acquistionlinerfi.it/web/error.html?_ncp=1753696951455.127431-1</t>
+          <t>https://www.acquistionlinerfi.it/esop/toolkit/opportunity/current/list.si?reset=true&amp;resetstored=true&amp;customLoginPage=%2Fweb%2Flogin.html&amp;_ncp=1781183967356.1684912-1#fh</t>
         </is>
       </c>
     </row>
@@ -899,17 +895,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>RETE FERROVIARIA ITALIANA</t>
+          <t>ACQUISTIONLINERFI</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>DAC.0374.2026 MDI_Isolatori per tirante a  terra per i sostegni di ormeggio tipo "LS-LSF-LSFP</t>
+          <t>DAC.0111.2026_Fornitura di SALDATURE ALLUMINOTERMICHE</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>30/06/2026</t>
+          <t>29/06/2026 12:00</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -924,12 +920,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Fornitura di isolatori per tirante a terra per i sostegni di ormeggio tipo "LS-LSF-LSFP".</t>
+          <t>Rete Ferroviaria Italiana</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://www.acquistionlinerfi.it/web/error.html?_ncp=1753696951455.127431-1</t>
+          <t>https://www.acquistionlinerfi.it/esop/toolkit/opportunity/current/list.si?reset=true&amp;resetstored=true&amp;customLoginPage=%2Fweb%2Flogin.html&amp;_ncp=1781183967356.1684912-1#fh</t>
         </is>
       </c>
     </row>
@@ -946,17 +942,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>RETE FERROVIARIA ITALIANA</t>
+          <t>ACQUISTIONLINERFI</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>DAC.0294.2026_Fornitura di MENSOLE IN ACCIAIO</t>
+          <t>DAC.0374.2026 MDI_Isolatori per tirante a  terra per i sostegni di ormeggio tipo "LS-LSF-LSFP</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>30/06/2026</t>
+          <t>30/06/2026 12:00</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -971,12 +967,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Fornitura di mensole in acciaio.</t>
+          <t>Rete Ferroviaria Italiana</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://www.acquistionlinerfi.it/web/error.html?_ncp=1753696951455.127431-1</t>
+          <t>https://www.acquistionlinerfi.it/esop/toolkit/opportunity/current/list.si?reset=true&amp;resetstored=true&amp;customLoginPage=%2Fweb%2Flogin.html&amp;_ncp=1781183967356.1684912-1#fh</t>
         </is>
       </c>
     </row>
@@ -993,17 +989,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>RETE FERROVIARIA ITALIANA</t>
+          <t>ACQUISTIONLINERFI</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>DAC.0337.2026_AQ Indagini  Geognostiche, Geofisiche, Geotecniche e sui Materiali</t>
+          <t>DAC.0294.2026_Fornitura di MENSOLE IN ACCIAIO</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>01/07/2026</t>
+          <t>30/06/2026 12:00</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1013,17 +1009,17 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Lavori</t>
+          <t>Fornitura</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Indagini Geognostiche, Geofisiche, Geotecniche e sui Materiali</t>
+          <t>Rete Ferroviaria Italiana</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://www.acquistionlinerfi.it/web/error.html?_ncp=1753696951455.127431-1</t>
+          <t>https://www.acquistionlinerfi.it/esop/toolkit/opportunity/current/list.si?reset=true&amp;resetstored=true&amp;customLoginPage=%2Fweb%2Flogin.html&amp;_ncp=1781183967356.1684912-1#fh</t>
         </is>
       </c>
     </row>
@@ -1040,17 +1036,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>RETE FERROVIARIA ITALIANA</t>
+          <t>ACQUISTIONLINERFI</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>DAC.0332.2026 - FORNITURA DI AGHI GREZZI CON FORGIATURA (Componenti per AdD +- 200)</t>
+          <t>DAC.0337.2026_AQ Indagini  Geognostiche, Geofisiche, Geotecniche e sui Materiali</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>02/07/2026</t>
+          <t>01/07/2026 12:00</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1060,17 +1056,17 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Fornitura</t>
+          <t>Lavori</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Fornitura di aghi grezzi con forgiatura (Componenti per AdD +- 200)</t>
+          <t>Rete Ferroviaria Italiana</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://www.acquistionlinerfi.it/web/error.html?_ncp=1753696951455.127431-1</t>
+          <t>https://www.acquistionlinerfi.it/esop/toolkit/opportunity/current/list.si?reset=true&amp;resetstored=true&amp;customLoginPage=%2Fweb%2Flogin.html&amp;_ncp=1781183967356.1684912-1#fh</t>
         </is>
       </c>
     </row>
@@ -1087,17 +1083,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>RETE FERROVIARIA ITALIANA</t>
+          <t>ACQUISTIONLINERFI</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>DAC.0254.2026 - FORNITURA DI BARRE DI COLLEGAMENTO AD U (Componenti per AdD +/- 200)</t>
+          <t>DAC.0332.2026 - FORNITURA DI AGHI GREZZI CON FORGIATURA (Componenti per AdD +- 200)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>03/07/2026</t>
+          <t>02/07/2026 12:00</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1112,12 +1108,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Fornitura di barre di collegamento ad U (Componenti per AdD +/- 200)</t>
+          <t>Rete Ferroviaria Italiana</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://www.acquistionlinerfi.it/web/error.html?_ncp=1753696951455.127431-1</t>
+          <t>https://www.acquistionlinerfi.it/esop/toolkit/opportunity/current/list.si?reset=true&amp;resetstored=true&amp;customLoginPage=%2Fweb%2Flogin.html&amp;_ncp=1781183967356.1684912-1#fh</t>
         </is>
       </c>
     </row>
@@ -1134,37 +1130,84 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>RETE FERROVIARIA ITALIANA</t>
+          <t>ACQUISTIONLINERFI</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
+          <t>DAC.0254.2026 - FORNITURA DI BARRE DI COLLEGAMENTO AD U (Componenti per AdD +/- 200)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>03/07/2026 12:00</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Fornitura</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Rete Ferroviaria Italiana</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://www.acquistionlinerfi.it/esop/toolkit/opportunity/current/list.si?reset=true&amp;resetstored=true&amp;customLoginPage=%2Fweb%2Flogin.html&amp;_ncp=1781183967356.1684912-1#fh</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>https://www.acquistionlinerfi.it/web/error.html?_ncp=1753696951455.127431-1</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ACQUISTIONLINERFI</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>DAC.0366.2026 - GPA- Fornitura con posa nr. due macchine fresatrici ONA Pontassieve</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>07/07/2026</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>07/07/2026 12:00</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
         <is>
           <t>Fornitura</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Fornitura con posa nr. due macchine fresatrici ONA Pontassieve</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>https://www.acquistionlinerfi.it/web/error.html?_ncp=1753696951455.127431-1</t>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Rete Ferroviaria Italiana</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://www.acquistionlinerfi.it/esop/toolkit/opportunity/current/list.si?reset=true&amp;resetstored=true&amp;customLoginPage=%2Fweb%2Flogin.html&amp;_ncp=1781183967356.1684912-1#fh</t>
         </is>
       </c>
     </row>

</xml_diff>